<commit_message>
Document corpus collection completeness
</commit_message>
<xml_diff>
--- a/data/output/anf_relatorio.xlsx
+++ b/data/output/anf_relatorio.xlsx
@@ -1381,7 +1381,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>http://www.anf-cinemateca.ro/: HTTPConnectionPool(host='www.anf-cinemateca.ro', port=80): Max retries exceeded with url: / (Caused by ConnectTimeoutError(&lt;HTTPConnection(host='www.anf-cinemateca.ro', port=80) at 0x1e5325265d0&gt;, 'Connection to www.anf-cinemateca.ro timed out. (connect timeout=8)'))</t>
+          <t>http://www.anf-cinemateca.ro/: HTTPConnectionPool(host='www.anf-cinemateca.ro', port=80): Max retries exceeded with url: / (Caused by ConnectTimeoutError(&lt;HTTPConnection(host='www.anf-cinemateca.ro', port=80) at 0x1b3dcf4b0d0&gt;, 'Connection to www.anf-cinemateca.ro timed out. (connect timeout=8)'))</t>
         </is>
       </c>
     </row>
@@ -2306,7 +2306,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>HTTPConnectionPool(host='www.anf-cinemateca.ro', port=80): Max retries exceeded with url: / (Caused by ConnectTimeoutError(&lt;HTTPConnection(host='www.anf-cinemateca.ro', port=80) at 0x1e5325265d0&gt;, 'Connection to www.anf-cinemateca.ro timed out. (connect timeout=8)'))</t>
+          <t>HTTPConnectionPool(host='www.anf-cinemateca.ro', port=80): Max retries exceeded with url: / (Caused by ConnectTimeoutError(&lt;HTTPConnection(host='www.anf-cinemateca.ro', port=80) at 0x1b3dcf4b0d0&gt;, 'Connection to www.anf-cinemateca.ro timed out. (connect timeout=8)'))</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3449,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>http://www.anf-cinemateca.ro/: HTTPConnectionPool(host='www.anf-cinemateca.ro', port=80): Max retries exceeded with url: / (Caused by ConnectTimeoutError(&lt;HTTPConnection(host='www.anf-cinemateca.ro', port=80) at 0x1e5325265d0&gt;, 'Connection to www.anf-cinemateca.ro timed out. (connect timeout=8)'))</t>
+          <t>http://www.anf-cinemateca.ro/: HTTPConnectionPool(host='www.anf-cinemateca.ro', port=80): Max retries exceeded with url: / (Caused by ConnectTimeoutError(&lt;HTTPConnection(host='www.anf-cinemateca.ro', port=80) at 0x1b3dcf4b0d0&gt;, 'Connection to www.anf-cinemateca.ro timed out. (connect timeout=8)'))</t>
         </is>
       </c>
       <c r="V2" t="n">

</xml_diff>

<commit_message>
Prepare Streamlit MVP deployment
</commit_message>
<xml_diff>
--- a/data/output/anf_relatorio.xlsx
+++ b/data/output/anf_relatorio.xlsx
@@ -546,7 +546,7 @@
   <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -565,7 +565,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Plataforma externa de exibição online</t>
+          <t>Streaming pago/autenticado em plataforma externa</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -586,7 +586,7 @@
   <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="47" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -605,7 +605,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Acesso mediado por plataforma externa de exibição online</t>
+          <t>Acesso pago/autenticado em plataforma externa</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1180,7 +1180,7 @@
     <col width="26" customWidth="1" min="18" max="18"/>
     <col width="17" customWidth="1" min="19" max="19"/>
     <col width="60" customWidth="1" min="20" max="20"/>
-    <col width="60" customWidth="1" min="21" max="21"/>
+    <col width="7" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1379,11 +1379,7 @@
           <t>Corpus institucional incorporado por superfície externa Cinemateca Online/Eventbook. A rota oficial anf-cinemateca.ro não respondeu nesta rodada; a coleta não representa catálogo total da ANF e não baixa mídia.</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>http://www.anf-cinemateca.ro/: HTTPConnectionPool(host='www.anf-cinemateca.ro', port=80): Max retries exceeded with url: / (Caused by ConnectTimeoutError(&lt;HTTPConnection(host='www.anf-cinemateca.ro', port=80) at 0x1b3dcf4b0d0&gt;, 'Connection to www.anf-cinemateca.ro timed out. (connect timeout=8)'))</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2145,7 +2141,7 @@
     <col width="19" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
     <col width="60" customWidth="1" min="16" max="16"/>
-    <col width="60" customWidth="1" min="17" max="17"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2284,15 +2280,17 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>http://www.anf-cinemateca.ro/</t>
+          <t>https://www.anf.gov.ro/</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>erro</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>200</v>
+      </c>
       <c r="N2" t="n">
         <v>0</v>
       </c>
@@ -2304,11 +2302,7 @@
           <t>Site oficial informado pela FIAF/EFG; indisponibilidade não bloqueia a rota externa validada.</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>HTTPConnectionPool(host='www.anf-cinemateca.ro', port=80): Max retries exceeded with url: / (Caused by ConnectTimeoutError(&lt;HTTPConnection(host='www.anf-cinemateca.ro', port=80) at 0x1b3dcf4b0d0&gt;, 'Connection to www.anf-cinemateca.ro timed out. (connect timeout=8)'))</t>
-        </is>
-      </c>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3200,15 +3194,15 @@
     <col width="26" customWidth="1" min="18" max="18"/>
     <col width="17" customWidth="1" min="19" max="19"/>
     <col width="60" customWidth="1" min="20" max="20"/>
-    <col width="60" customWidth="1" min="21" max="21"/>
+    <col width="7" customWidth="1" min="21" max="21"/>
     <col width="29" customWidth="1" min="22" max="22"/>
     <col width="30" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="21" customWidth="1" min="25" max="25"/>
     <col width="45" customWidth="1" min="26" max="26"/>
     <col width="24" customWidth="1" min="27" max="27"/>
-    <col width="39" customWidth="1" min="28" max="28"/>
-    <col width="58" customWidth="1" min="29" max="29"/>
+    <col width="50" customWidth="1" min="28" max="28"/>
+    <col width="47" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3447,11 +3441,7 @@
           <t>Corpus institucional incorporado por superfície externa Cinemateca Online/Eventbook. A rota oficial anf-cinemateca.ro não respondeu nesta rodada; a coleta não representa catálogo total da ANF e não baixa mídia.</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>http://www.anf-cinemateca.ro/: HTTPConnectionPool(host='www.anf-cinemateca.ro', port=80): Max retries exceeded with url: / (Caused by ConnectTimeoutError(&lt;HTTPConnection(host='www.anf-cinemateca.ro', port=80) at 0x1b3dcf4b0d0&gt;, 'Connection to www.anf-cinemateca.ro timed out. (connect timeout=8)'))</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="n">
         <v>8</v>
       </c>
@@ -3480,12 +3470,12 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>Plataforma externa de exibição online</t>
+          <t>Streaming pago/autenticado em plataforma externa</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>Acesso mediado por plataforma externa de exibição online</t>
+          <t>Acesso pago/autenticado em plataforma externa</t>
         </is>
       </c>
     </row>
@@ -3522,7 +3512,7 @@
     <col width="54" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
     <col width="35" customWidth="1" min="19" max="19"/>
-    <col width="39" customWidth="1" min="20" max="20"/>
+    <col width="50" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3721,7 +3711,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Plataforma externa de exibição online</t>
+          <t>Streaming pago/autenticado em plataforma externa</t>
         </is>
       </c>
     </row>
@@ -3819,7 +3809,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Plataforma externa de exibição online</t>
+          <t>Streaming pago/autenticado em plataforma externa</t>
         </is>
       </c>
     </row>
@@ -3917,7 +3907,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Plataforma externa de exibição online</t>
+          <t>Streaming pago/autenticado em plataforma externa</t>
         </is>
       </c>
     </row>
@@ -4011,7 +4001,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Plataforma externa de exibição online</t>
+          <t>Streaming pago/autenticado em plataforma externa</t>
         </is>
       </c>
     </row>
@@ -4109,7 +4099,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Plataforma externa de exibição online</t>
+          <t>Streaming pago/autenticado em plataforma externa</t>
         </is>
       </c>
     </row>
@@ -4207,7 +4197,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Plataforma externa de exibição online</t>
+          <t>Streaming pago/autenticado em plataforma externa</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4291,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Plataforma externa de exibição online</t>
+          <t>Streaming pago/autenticado em plataforma externa</t>
         </is>
       </c>
     </row>
@@ -4399,7 +4389,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Plataforma externa de exibição online</t>
+          <t>Streaming pago/autenticado em plataforma externa</t>
         </is>
       </c>
     </row>

</xml_diff>